<commit_message>
Auto update nse_indices_1 outputs
</commit_message>
<xml_diff>
--- a/nse_indices_1_dashboard.xlsx
+++ b/nse_indices_1_dashboard.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>3.35%</t>
+          <t>3.34%</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>4.03</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="7">
@@ -791,7 +791,7 @@
         <v>22866.5</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>16.53000068664551</v>
+        <v>16.51000022888184</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>22866.5</v>
@@ -15750,7 +15750,7 @@
         <v>0.2</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>4.03</v>
+        <v>3.9</v>
       </c>
       <c r="K2" s="4" t="n">
         <v>0.2</v>
@@ -30721,7 +30721,7 @@
         <v>-0.37</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>0</v>
+        <v>-0.12</v>
       </c>
       <c r="K2" s="4" t="n">
         <v>-0.37</v>

</xml_diff>